<commit_message>
2026-09-01: Provide release of current third project
</commit_message>
<xml_diff>
--- a/2026-09-01/problems/result.xlsx
+++ b/2026-09-01/problems/result.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30015"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\【】理工大\【02】数学建模\2026\省赛出题\多源异质定位数据融合\更新\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\第3轮集训题目\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38DB44E1-A924-4996-81CE-10C837096C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C063C7-3046-4552-888F-C33210670502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="38">
   <si>
     <t>目标编号</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -59,6 +59,95 @@
   </si>
   <si>
     <t>任务执行时刻(s)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>P03</t>
+  </si>
+  <si>
+    <t>P11</t>
+  </si>
+  <si>
+    <t>P17</t>
+  </si>
+  <si>
+    <t>P18</t>
+  </si>
+  <si>
+    <t>P15</t>
+  </si>
+  <si>
+    <t>P16</t>
+  </si>
+  <si>
+    <t>P13</t>
+  </si>
+  <si>
+    <t>S06</t>
+  </si>
+  <si>
+    <t>P12</t>
+  </si>
+  <si>
+    <t>P07</t>
+  </si>
+  <si>
+    <t>S08</t>
+  </si>
+  <si>
+    <t>P09</t>
+  </si>
+  <si>
+    <t>P05</t>
+  </si>
+  <si>
+    <t>S09</t>
+  </si>
+  <si>
+    <t>P08</t>
+  </si>
+  <si>
+    <t>P14</t>
+  </si>
+  <si>
+    <t>P04</t>
+  </si>
+  <si>
+    <t>S05</t>
+  </si>
+  <si>
+    <t>S04</t>
+  </si>
+  <si>
+    <t>P06</t>
+  </si>
+  <si>
+    <t>P02</t>
+  </si>
+  <si>
+    <t>P10</t>
+  </si>
+  <si>
+    <t>S12</t>
+  </si>
+  <si>
+    <t>S10</t>
+  </si>
+  <si>
+    <t>S13</t>
+  </si>
+  <si>
+    <t>S11</t>
+  </si>
+  <si>
+    <t>拍照</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>射击</t>
+  </si>
+  <si>
+    <t>射击</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -125,11 +214,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -410,7 +502,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="15.77734375" customWidth="1"/>
@@ -447,6 +539,18 @@
       <c r="A2">
         <v>1</v>
       </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="4">
+        <v>446.2</v>
+      </c>
+      <c r="E2" s="4">
+        <v>446.7</v>
+      </c>
       <c r="H2" s="1" t="s">
         <v>4</v>
       </c>
@@ -459,6 +563,18 @@
       <c r="A3">
         <v>2</v>
       </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="4">
+        <v>446.7</v>
+      </c>
+      <c r="E3" s="4">
+        <v>447.2</v>
+      </c>
       <c r="H3" s="2" t="s">
         <v>1</v>
       </c>
@@ -479,6 +595,18 @@
       <c r="A4">
         <v>3</v>
       </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="4">
+        <v>447.2</v>
+      </c>
+      <c r="E4" s="4">
+        <v>447.7</v>
+      </c>
       <c r="H4" s="2">
         <v>1</v>
       </c>
@@ -498,6 +626,18 @@
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="4">
+        <v>447.7</v>
+      </c>
+      <c r="E5" s="4">
+        <v>448.2</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -509,29 +649,498 @@
       <c r="A6">
         <v>5</v>
       </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="4">
+        <v>448.2</v>
+      </c>
+      <c r="E6" s="4">
+        <v>448.7</v>
+      </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="4">
+        <v>448.7</v>
+      </c>
+      <c r="E7" s="4">
+        <v>449.2</v>
+      </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="4">
+        <v>449.4</v>
+      </c>
+      <c r="E8" s="4">
+        <v>449.9</v>
+      </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="4">
+        <v>449.9</v>
+      </c>
+      <c r="E9" s="4">
+        <v>451.4</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="4">
+        <v>451.4</v>
+      </c>
+      <c r="E10" s="4">
+        <v>451.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="4">
+        <v>457.7</v>
+      </c>
+      <c r="E11" s="4">
+        <v>458.2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="4">
+        <v>458.7</v>
+      </c>
+      <c r="E12" s="4">
+        <v>460.2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="4">
+        <v>460.2</v>
+      </c>
+      <c r="E13" s="4">
+        <v>460.7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="4">
+        <v>460.7</v>
+      </c>
+      <c r="E14" s="4">
+        <v>461.2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="4">
+        <v>461.2</v>
+      </c>
+      <c r="E15" s="4">
+        <v>462.7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="4">
+        <v>462.7</v>
+      </c>
+      <c r="E16" s="4">
+        <v>463.2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="4">
+        <v>463.2</v>
+      </c>
+      <c r="E17" s="4">
+        <v>463.7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="4">
+        <v>463.7</v>
+      </c>
+      <c r="E18" s="4">
+        <v>464.2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="4">
+        <v>464.2</v>
+      </c>
+      <c r="E19" s="4">
+        <v>465.7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="4">
+        <v>465.7</v>
+      </c>
+      <c r="E20" s="4">
+        <v>467.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" s="4">
+        <v>467.2</v>
+      </c>
+      <c r="E21" s="4">
+        <v>467.7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22" s="4">
+        <v>476.8</v>
+      </c>
+      <c r="E22" s="4">
+        <v>477.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" s="4">
+        <v>477.4</v>
+      </c>
+      <c r="E23" s="4">
+        <v>477.9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" s="4">
+        <v>493</v>
+      </c>
+      <c r="E24" s="4">
+        <v>493.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="4">
+        <v>493.6</v>
+      </c>
+      <c r="E25" s="4">
+        <v>494.1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26" s="4">
+        <v>494.1</v>
+      </c>
+      <c r="E26" s="4">
+        <v>494.6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D27" s="4">
+        <v>506.7</v>
+      </c>
+      <c r="E27" s="4">
+        <v>507.2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28" s="4">
+        <v>515.20000000000005</v>
+      </c>
+      <c r="E28" s="4">
+        <v>515.70000000000005</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" s="4">
+        <v>516.20000000000005</v>
+      </c>
+      <c r="E29" s="4">
+        <v>517.70000000000005</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>32</v>
+      </c>
+      <c r="C30" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" s="4">
+        <v>533.6</v>
+      </c>
+      <c r="E30" s="4">
+        <v>535.1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31" s="4">
+        <v>749.9</v>
+      </c>
+      <c r="E31" s="4">
+        <v>750.4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" t="s">
+        <v>35</v>
+      </c>
+      <c r="D32" s="4">
+        <v>750.8</v>
+      </c>
+      <c r="E32" s="4">
+        <v>751.3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>33</v>
+      </c>
+      <c r="C33" t="s">
+        <v>36</v>
+      </c>
+      <c r="D33" s="4">
+        <v>762.7</v>
+      </c>
+      <c r="E33" s="4">
+        <v>764.2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>34</v>
+      </c>
+      <c r="C34" t="s">
+        <v>36</v>
+      </c>
+      <c r="D34" s="4">
+        <v>775.7</v>
+      </c>
+      <c r="E34" s="4">
+        <v>777.2</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>